<commit_message>
Add embedded charts (line/pie/bar/doughnut) to trade log; fix crypto order time-in-force bug
</commit_message>
<xml_diff>
--- a/trades.xlsx
+++ b/trades.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Trades" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Charts" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -123,6 +124,434 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Cumulative P&amp;L Over Time</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Trades'!L1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <val>
+            <numRef>
+              <f>'Trades'!$L$2:$L$100000</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Trade #</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>P&amp;L ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Win / Loss Distribution</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Summary'!$A$3:$A$4</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Summary'!$B$3:$B$4</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Realized P&amp;L by Symbol</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Charts'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$A$2:$A$201</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$B$2:$B$201</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Symbol</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>P&amp;L ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Trades by Asset Class</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <doughnutChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Charts'!E1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Charts'!$D$2:$D$3</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Charts'!$E$2:$E$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+        <holeSize val="10"/>
+      </doughnutChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8640000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -414,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,11 +902,16 @@
           <t>Order ID</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Cumulative P&amp;L ($)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-21 20:54:25</t>
+          <t>2026-07-21 21:00:25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -513,12 +947,15 @@
         <is>
           <t>3feaa311-3cb7-40a9-bc26-a494cb4f7e35</t>
         </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-21 20:54:34</t>
+          <t>2026-07-21 21:00:25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -560,6 +997,53 @@
         <is>
           <t>4b6a43fd-d304-4527-a994-1180d972aedb</t>
         </is>
+      </c>
+      <c r="L3" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-21 21:01:43</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL/USD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>crypto</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>351.210888</v>
+      </c>
+      <c r="F4" t="n">
+        <v>78.073589</v>
+      </c>
+      <c r="G4" t="n">
+        <v>27420.29</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>RSI bounced from 38.6→41.3 (oversold rebound); news: "Bitcoin Tops $66,000 As Ethereum, XRP, Dogecoin Rally On White House Backing CLARITY Act Ethics Package" (sentiment=+2)</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1e8c7626-0008-4f69-adb4-45a07637504d</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>-0.03</v>
       </c>
     </row>
   </sheetData>
@@ -646,4 +1130,267 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E201"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total Realized P&amp;L ($)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Asset Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Trade Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>crypto</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix crypto position sizing to respect non-marginable buying power
</commit_message>
<xml_diff>
--- a/trades.xlsx
+++ b/trades.xlsx
@@ -843,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1043,6 +1043,94 @@
         </is>
       </c>
       <c r="L4" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-21 21:15:16</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>GOOGL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>27</v>
+      </c>
+      <c r="F5" t="n">
+        <v>349.7</v>
+      </c>
+      <c r="G5" t="n">
+        <v>9441.9</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>RSI bounced from 35.5→49.4 (oversold rebound); news: "Intel Stock Surges 5%: Memory Upgrade and Google AI Deal Fuel Rally" (sentiment=+7)</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>69ec3278-39e8-483d-ab6d-38f3fb029a7a</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>-0.03</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-21 21:15:17</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AMZN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>stock</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>33</v>
+      </c>
+      <c r="F6" t="n">
+        <v>247.79</v>
+      </c>
+      <c r="G6" t="n">
+        <v>8177.07</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>RSI bounced from 38.6→44.2 (oversold rebound); news: "Micron Leads Memory-Stock Rally, Nasdaq 100 Tops 29,000: Stock Market Today" (sentiment=+1)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>19229d7d-2069-479c-80f7-c0f89162e8b9</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
         <v>-0.03</v>
       </c>
     </row>
@@ -1178,7 +1266,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Fix: skip stock stop-loss/take-profit checks outside market hours; only log actually-filled orders; reconcile missed SOL/USD sell
</commit_message>
<xml_diff>
--- a/trades.xlsx
+++ b/trades.xlsx
@@ -843,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1132,6 +1132,56 @@
       </c>
       <c r="L6" t="n">
         <v>-0.03</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-22 08:53:04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SOL/USD</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>crypto</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>350.33286078</v>
+      </c>
+      <c r="F7" t="n">
+        <v>76.75501300000001</v>
+      </c>
+      <c r="G7" t="n">
+        <v>26889.8</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>stop-loss/take-profit sweep (reconciled — this sell executed on Alpaca but was missed by a since-fixed logging bug)</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>-461.94</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-1.6889</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>85684ddc-2134-4edc-bfb8-0d5087fb527d</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>-461.97</v>
       </c>
     </row>
   </sheetData>
@@ -1226,7 +1276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1270,213 +1320,23 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SOL/USD</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-461.94</v>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>crypto</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>

<commit_message>
Fix phantom blank row in EquityLog on fresh workbook creation
_style_header set freeze_panes via ws.cell(row+1, 1), which implicitly
creates that row in the sheet's dimensions even though no value is
written. On a brand-new EquityLog sheet (header row only, no data yet),
that touch inserted an empty row 2 before the first real snapshot ever
got appended, pushing it to row 3. Positions self-healed via its
delete_rows call; Trades/Summary/Dashboard were unaffected because they
write real data before calling _style_header. Use a string coordinate
for freeze_panes instead, which doesn't touch worksheet dimensions.
Also removes the one stray blank row already written to trades.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/trades.xlsx
+++ b/trades.xlsx
@@ -2453,7 +2453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E201"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2574,198 +2574,6 @@
         <v>-776</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
-    <row r="201"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3023,7 +2831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -3096,77 +2904,77 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-23 17:17:45</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>528</v>
+      </c>
+      <c r="C2" t="n">
+        <v>528</v>
+      </c>
+      <c r="D2" t="n">
+        <v>528</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>528</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-23 17:17:45</t>
+          <t>2026-07-23 17:28:39</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>528</v>
+        <v>522.9299999999999</v>
       </c>
       <c r="C3" t="n">
-        <v>528</v>
+        <v>268.07</v>
       </c>
       <c r="D3" t="n">
-        <v>528</v>
+        <v>268.07</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>-5.07</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>-0.9602000000000001</v>
       </c>
       <c r="G3" t="n">
         <v>528</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>-0.9602000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>254.86</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-07-23 17:28:39</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>522.9299999999999</v>
-      </c>
-      <c r="C4" t="n">
-        <v>268.07</v>
-      </c>
-      <c r="D4" t="n">
-        <v>268.07</v>
-      </c>
-      <c r="E4" t="n">
-        <v>-5.07</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-0.9602000000000001</v>
-      </c>
-      <c r="G4" t="n">
-        <v>528</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-0.9602000000000001</v>
-      </c>
-      <c r="I4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J4" t="n">
-        <v>254.86</v>
-      </c>
-      <c r="K4" t="n">
         <v>48.7378</v>
       </c>
     </row>

</xml_diff>